<commit_message>
scan: seg6 2026-07-16 18:17 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-07-16.xlsx
+++ b/output/full_scan/batch_seq7_2026-07-16.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O127"/>
+  <dimension ref="A1:O128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3866,21 +3866,21 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6679</v>
+        <v>6831</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>鈺太</t>
+          <t>邁科</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>337.3494967727941</v>
+        <v>339.9747140453296</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>239</v>
+        <v>680</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>34.45564610570626</v>
+        <v>40.88760255231058</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>25.23223395783102</v>
+        <v>23.35414615265801</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.5595092790651596</v>
+        <v>0.1798807287223325</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-2.037149414544889</v>
+        <v>-26.30608983523077</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3919,21 +3919,21 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6568</v>
+        <v>6679</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>宏觀</t>
+          <t>鈺太</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>335.3364462634262</v>
+        <v>337.3494967727941</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>151</v>
+        <v>239</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,16 +3944,16 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>32.20921357302338</v>
+        <v>34.45564610570626</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>40.76682660104276</v>
+        <v>25.23223395783102</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.4276397165704528</v>
+        <v>0.5595092790651596</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.8972728995583239</v>
+        <v>-2.037149414544889</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6669</v>
+        <v>6568</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>緯穎</t>
+          <t>宏觀</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>331.5585480537792</v>
+        <v>335.3364462634262</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>5115</v>
+        <v>151</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>54.0469409718479</v>
+        <v>32.20921357302338</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>11.20984866717954</v>
+        <v>40.76682660104276</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.3857297978587333</v>
+        <v>0.4276397165704528</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>26.41086708471664</v>
+        <v>0.8972728995583239</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6770</v>
+        <v>6669</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>力積電</t>
+          <t>緯穎</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>327.6956103236068</v>
+        <v>331.5585480537792</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>76.5</v>
+        <v>5115</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>54.73001965129223</v>
+        <v>54.0469409718479</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>14.47584011895334</v>
+        <v>11.20984866717954</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>1.840949221424594</v>
+        <v>0.3857297978587333</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.3961997336644529</v>
+        <v>26.41086708471664</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6706</v>
+        <v>6770</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>惠特</t>
+          <t>力積電</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>326.7704208743225</v>
+        <v>327.6956103236068</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>122</v>
+        <v>76.5</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>31.1461149068598</v>
+        <v>54.73001965129223</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>21.28292928379147</v>
+        <v>14.47584011895334</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.5174998384296311</v>
+        <v>1.840949221424594</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-2.214768414630626</v>
+        <v>-0.3961997336644529</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6625</v>
+        <v>6706</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>必應</t>
+          <t>惠特</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>325.6889764578236</v>
+        <v>326.7704208743225</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>78.59999999999999</v>
+        <v>122</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>54.12828627322428</v>
+        <v>31.1461149068598</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>21.58538909969617</v>
+        <v>21.28292928379147</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.8805398927881471</v>
+        <v>0.5174998384296311</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.2075595156156993</v>
+        <v>-2.214768414630626</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6722</v>
+        <v>6625</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>輝創</t>
+          <t>必應</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>323.2818805350968</v>
+        <v>325.6889764578236</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>34.45</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>38.62850389268254</v>
+        <v>54.12828627322428</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>39.64965388022912</v>
+        <v>21.58538909969617</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.6427415277652583</v>
+        <v>0.8805398927881471</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.01746152495041</v>
+        <v>-0.2075595156156993</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6670</v>
+        <v>6722</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>復盛應用</t>
+          <t>輝創</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>321.310198884349</v>
+        <v>323.2818805350968</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>263</v>
+        <v>34.45</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>49.42465931505083</v>
+        <v>38.62850389268254</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>14.87375882180444</v>
+        <v>39.64965388022912</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.5161988043574582</v>
+        <v>0.6427415277652583</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.5367961690226473</v>
+        <v>0.01746152495041</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6742</v>
+        <v>6670</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>澤米</t>
+          <t>復盛應用</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>318.0634125976003</v>
+        <v>321.310198884349</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>51</v>
+        <v>263</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>34.07185749261772</v>
+        <v>49.42465931505083</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>22.54476451611669</v>
+        <v>14.87375882180444</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.1135607067011274</v>
+        <v>0.5161988043574582</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-2.160745861723234</v>
+        <v>0.5367961690226473</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6532</v>
+        <v>6742</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>瑞耘</t>
+          <t>澤米</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>317.3682545167957</v>
+        <v>318.0634125976003</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>73.90000000000001</v>
+        <v>51</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>30.39477742812683</v>
+        <v>34.07185749261772</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>21.90624280033299</v>
+        <v>22.54476451611669</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.3794468405879679</v>
+        <v>0.1135607067011274</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-1.40986327297176</v>
+        <v>-2.160745861723234</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6643</v>
+        <v>6532</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>M31</t>
+          <t>瑞耘</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>309.6569712207369</v>
+        <v>317.3682545167957</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>412</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>31.44065083676832</v>
+        <v>30.39477742812683</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>22.05753695941272</v>
+        <v>21.90624280033299</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.8653796303819269</v>
+        <v>0.3794468405879679</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-4.291317680720589</v>
+        <v>-1.40986327297176</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6641</v>
+        <v>6643</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>基士德-KY</t>
+          <t>M31</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>308.2704647902301</v>
+        <v>309.6569712207369</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>18</v>
+        <v>412</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>43.63061983730508</v>
+        <v>31.44065083676832</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>18.09382672390248</v>
+        <v>22.05753695941272</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.148832002130065</v>
+        <v>0.8653796303819269</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.0419175369575498</v>
+        <v>-4.291317680720589</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6556</v>
+        <v>6641</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>勝品</t>
+          <t>基士德-KY</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>303.829188316862</v>
+        <v>308.2704647902301</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>65.2</v>
+        <v>18</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>27.14516550843694</v>
+        <v>43.63061983730508</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>27.08753586854879</v>
+        <v>18.09382672390248</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.6428058678715973</v>
+        <v>0.148832002130065</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.8427486505365587</v>
+        <v>-0.0419175369575498</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6504</v>
+        <v>6556</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>南六</t>
+          <t>勝品</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>302.9031576446708</v>
+        <v>303.829188316862</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>36.3</v>
+        <v>65.2</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>49.18225280290204</v>
+        <v>27.14516550843694</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>13.60700960131659</v>
+        <v>27.08753586854879</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>2.160315820812746</v>
+        <v>0.6428058678715973</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.1253323709361912</v>
+        <v>-0.8427486505365587</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6526</v>
+        <v>6504</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>達發</t>
+          <t>南六</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>301.9635381038999</v>
+        <v>302.9031576446708</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>619</v>
+        <v>36.3</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,13 +4633,13 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>41.46212487278314</v>
+        <v>49.18225280290204</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>11.38430648088001</v>
+        <v>13.60700960131659</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.7099917406156385</v>
+        <v>2.160315820812746</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-6.465162304952668</v>
+        <v>0.1253323709361912</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6803</v>
+        <v>6526</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>崑鼎</t>
+          <t>達發</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>297.825318004729</v>
+        <v>301.9635381038999</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>272</v>
+        <v>619</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>29.4287378900617</v>
+        <v>41.46212487278314</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>43.48987091009037</v>
+        <v>11.38430648088001</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.4845596214913797</v>
+        <v>0.7099917406156385</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-1.397636092196548</v>
+        <v>-6.465162304952668</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6591</v>
+        <v>6803</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>動力-KY</t>
+          <t>崑鼎</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>294.3718437127364</v>
+        <v>297.825318004729</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>45.35</v>
+        <v>272</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>23.7504768059932</v>
+        <v>29.4287378900617</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>32.05769641762278</v>
+        <v>43.48987091009037</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.6998676849684365</v>
+        <v>0.4845596214913797</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.9163798734426279</v>
+        <v>-1.397636092196548</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4767,21 +4767,21 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6776</v>
+        <v>6591</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>展碁國際</t>
+          <t>動力-KY</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>292.8455462059765</v>
+        <v>294.3718437127364</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>55.4</v>
+        <v>45.35</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>44.86287807768795</v>
+        <v>23.7504768059932</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>14.62093647290292</v>
+        <v>32.05769641762278</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.2737084530654473</v>
+        <v>0.6998676849684365</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.1312087499120193</v>
+        <v>-0.9163798734426279</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6541</v>
+        <v>6776</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>泰福-KY</t>
+          <t>展碁國際</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>284.5233565237392</v>
+        <v>292.8455462059765</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>40.3</v>
+        <v>55.4</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>48.67948794057429</v>
+        <v>44.86287807768795</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>15.16950082247098</v>
+        <v>14.62093647290292</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.5790545593727386</v>
+        <v>0.2737084530654473</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-0.1320916265067105</v>
+        <v>0.1312087499120193</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6756</v>
+        <v>6541</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>威鋒電子</t>
+          <t>泰福-KY</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>273.2777828177825</v>
+        <v>284.5233565237392</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>96</v>
+        <v>40.3</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>46.57157620695239</v>
+        <v>48.67948794057429</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>16.32172622428492</v>
+        <v>15.16950082247098</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.5166652694560016</v>
+        <v>0.5790545593727386</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.3715633147028885</v>
+        <v>-0.1320916265067105</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6821</v>
+        <v>6756</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>聯寶</t>
+          <t>威鋒電子</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>273.2365528872714</v>
+        <v>273.2777828177825</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>48.1</v>
+        <v>96</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>29.47128913067638</v>
+        <v>46.57157620695239</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>19.37605966909245</v>
+        <v>16.32172622428492</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.1603978052888555</v>
+        <v>0.5166652694560016</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-1.491951651018011</v>
+        <v>-0.3715633147028885</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6840</v>
+        <v>6821</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>東研信超</t>
+          <t>聯寶</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>270.3223255052202</v>
+        <v>273.2365528872714</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>62.1</v>
+        <v>48.1</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>43.46856426085931</v>
+        <v>29.47128913067638</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>10.99166609077953</v>
+        <v>19.37605966909245</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.1577518644769982</v>
+        <v>0.1603978052888555</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.2294923802190762</v>
+        <v>-1.491951651018011</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6531</v>
+        <v>6840</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>愛普*</t>
+          <t>東研信超</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>269.6480263963092</v>
+        <v>270.3223255052202</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>909</v>
+        <v>62.1</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>45.68865701286615</v>
+        <v>43.46856426085931</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>16.00897510072802</v>
+        <v>10.99166609077953</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.9051647789659582</v>
+        <v>0.1577518644769982</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-9.59285081854992</v>
+        <v>-0.2294923802190762</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6823</v>
+        <v>6531</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>濾能</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>265.7664666352802</v>
+        <v>269.6480263963092</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>68.3</v>
+        <v>909</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>47.25934478736312</v>
+        <v>45.68865701286615</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>13.27226426134484</v>
+        <v>16.00897510072802</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.7512629903948266</v>
+        <v>0.9051647789659582</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.2622379669869263</v>
+        <v>-9.59285081854992</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6498</v>
+        <v>6823</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>久禾光</t>
+          <t>濾能</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>264.9616975893231</v>
+        <v>265.7664666352802</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>85</v>
+        <v>68.3</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>33.25347175180362</v>
+        <v>47.25934478736312</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>22.58447760409513</v>
+        <v>13.27226426134484</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.3725400050936243</v>
+        <v>0.7512629903948266</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.9735532620207294</v>
+        <v>0.2622379669869263</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6835</v>
+        <v>6498</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>圓裕</t>
+          <t>久禾光</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>262.29678138283</v>
+        <v>264.9616975893231</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>32.65</v>
+        <v>85</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,16 +5216,16 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>25.90173683589797</v>
+        <v>33.25347175180362</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>32.19983148354292</v>
+        <v>22.58447760409513</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>1.1778383910942</v>
+        <v>0.3725400050936243</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.1892738062511177</v>
+        <v>-0.9735532620207294</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6788</v>
+        <v>6835</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>華景電</t>
+          <t>圓裕</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>261.5480782317076</v>
+        <v>262.29678138283</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>384</v>
+        <v>32.65</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,49 +5269,49 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>39.73170116131034</v>
+        <v>25.90173683589797</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>14.9206105154177</v>
+        <v>32.19983148354292</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.3982841236767879</v>
+        <v>1.1778383910942</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L91" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M91" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-6.107528017010115</v>
+        <v>-0.1892738062511177</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6761</v>
+        <v>6788</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>穩得</t>
+          <t>華景電</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>259.3632683875211</v>
+        <v>261.5480782317076</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>167.5</v>
+        <v>384</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,25 +5322,25 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>37.38033668220066</v>
+        <v>39.73170116131034</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>15.06654762279232</v>
+        <v>14.9206105154177</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.2253924221841101</v>
+        <v>0.3982841236767879</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L92" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M92" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-2.48988649312268</v>
+        <v>-6.107528017010115</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5350,21 +5350,21 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6561</v>
+        <v>6761</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>是方</t>
+          <t>穩得</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>257.635118176102</v>
+        <v>259.3632683875211</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>323.5</v>
+        <v>167.5</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,16 +5375,16 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>35.70062695075339</v>
+        <v>37.38033668220066</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>24.11431268999592</v>
+        <v>15.06654762279232</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.2114024490733202</v>
+        <v>0.2253924221841101</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.929018089729344</v>
+        <v>-2.48988649312268</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6668</v>
+        <v>6561</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>中揚光</t>
+          <t>是方</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>250.4793872440776</v>
+        <v>257.635118176102</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>36</v>
+        <v>323.5</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>38.75614363652983</v>
+        <v>35.70062695075339</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>16.58423807612978</v>
+        <v>24.11431268999592</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.1744089160534973</v>
+        <v>0.2114024490733202</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.5012115252304299</v>
+        <v>-0.929018089729344</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6624</v>
+        <v>6668</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>萬年清</t>
+          <t>中揚光</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>244.1984729245421</v>
+        <v>250.4793872440776</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>44.45</v>
+        <v>36</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>52.6978895581486</v>
+        <v>38.75614363652983</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>7.161023242046273</v>
+        <v>16.58423807612978</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.1182985836776577</v>
+        <v>0.1744089160534973</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.6235937865386723</v>
+        <v>-0.5012115252304299</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6741</v>
+        <v>6624</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>91APP*-KY</t>
+          <t>萬年清</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>241.3967548298978</v>
+        <v>244.1984729245421</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>58.5</v>
+        <v>44.45</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>38.538052034734</v>
+        <v>52.6978895581486</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>16.74583633346862</v>
+        <v>7.161023242046273</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.6562865784725997</v>
+        <v>0.1182985836776577</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.2573058642639626</v>
+        <v>0.6235937865386723</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6698</v>
+        <v>6741</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>旭暉應材</t>
+          <t>91APP*-KY</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>238.1416643548432</v>
+        <v>241.3967548298978</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>38.4</v>
+        <v>58.5</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>43.65509766605599</v>
+        <v>38.538052034734</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>22.60936687386752</v>
+        <v>16.74583633346862</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.3288831103505301</v>
+        <v>0.6562865784725997</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.7466619878238284</v>
+        <v>-0.2573058642639626</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6794</v>
+        <v>6698</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>向榮生技-創</t>
+          <t>旭暉應材</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>236.383495245701</v>
+        <v>238.1416643548432</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>78.3</v>
+        <v>38.4</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>44.19547763973116</v>
+        <v>43.65509766605599</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>16.05059368081879</v>
+        <v>22.60936687386752</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.3324598172976021</v>
+        <v>0.3288831103505301</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.1701383146979036</v>
+        <v>-0.7466619878238284</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6708</v>
+        <v>6794</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>天擎</t>
+          <t>向榮生技-創</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>236.3188428726526</v>
+        <v>236.383495245701</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>38.75</v>
+        <v>78.3</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>43.67024279225826</v>
+        <v>44.19547763973116</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>16.73683272955298</v>
+        <v>16.05059368081879</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.3259294637008161</v>
+        <v>0.3324598172976021</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.0721394295388092</v>
+        <v>-0.1701383146979036</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6512</v>
+        <v>6708</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>啟發電</t>
+          <t>天擎</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>235.4993168590074</v>
+        <v>236.3188428726526</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>20.05</v>
+        <v>38.75</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>52.85742260548782</v>
+        <v>43.67024279225826</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>10.94724500964836</v>
+        <v>16.73683272955298</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.6626155757983424</v>
+        <v>0.3259294637008161</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.7879838916629762</v>
+        <v>-0.0721394295388092</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6781</v>
+        <v>6512</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>AES-KY</t>
+          <t>啟發電</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>233.1529914909032</v>
+        <v>235.4993168590074</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>1045</v>
+        <v>20.05</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>38.21180240280869</v>
+        <v>52.85742260548782</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>13.37772438887556</v>
+        <v>10.94724500964836</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.5154217627793373</v>
+        <v>0.6626155757983424</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-17.2517546032413</v>
+        <v>-0.7879838916629762</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6754</v>
+        <v>6781</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>匯僑設計</t>
+          <t>AES-KY</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>232.1945841777321</v>
+        <v>233.1529914909032</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>42.45</v>
+        <v>1045</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>42.13841144707701</v>
+        <v>38.21180240280869</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>16.1777353632258</v>
+        <v>13.37772438887556</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.4560639441718683</v>
+        <v>0.5154217627793373</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.1673818196822726</v>
+        <v>-17.2517546032413</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6592</v>
+        <v>6754</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>和潤企業</t>
+          <t>匯僑設計</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>225.876839552251</v>
+        <v>232.1945841777321</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>61.9</v>
+        <v>42.45</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>50.16833408270992</v>
+        <v>42.13841144707701</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>22.98597535529228</v>
+        <v>16.1777353632258</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.7376394298547825</v>
+        <v>0.4560639441718683</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.1180120711672362</v>
+        <v>-0.1673818196822726</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6768</v>
+        <v>6592</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>志強-KY</t>
+          <t>和潤企業</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>224.0522652000046</v>
+        <v>225.876839552251</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>71</v>
+        <v>61.9</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>28.31496921326621</v>
+        <v>50.16833408270992</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>32.02959075809282</v>
+        <v>22.98597535529228</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>1.275992534109559</v>
+        <v>0.7376394298547825</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.3480179275195585</v>
+        <v>-0.1180120711672362</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6581</v>
+        <v>6768</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>鋼聯</t>
+          <t>志強-KY</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>220.0735750261626</v>
+        <v>224.0522652000046</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>108</v>
+        <v>71</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>52.57611772287481</v>
+        <v>28.31496921326621</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>9.575515718327209</v>
+        <v>32.02959075809282</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>1.225577719328559</v>
+        <v>1.275992534109559</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.179680800293091</v>
+        <v>-0.3480179275195585</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>6792</v>
+        <v>6581</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>詠業</t>
+          <t>鋼聯</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>212.3570443588801</v>
+        <v>220.0735750261626</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>56.9</v>
+        <v>108</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>34.21039601143217</v>
+        <v>52.57611772287481</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>18.25657600591554</v>
+        <v>9.575515718327209</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.5235182400078677</v>
+        <v>1.225577719328559</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.9161225546766618</v>
+        <v>0.179680800293091</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6092,21 +6092,21 @@
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6667</v>
+        <v>6792</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>信紘科</t>
+          <t>詠業</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>210.7657977737905</v>
+        <v>212.3570443588801</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>257.5</v>
+        <v>56.9</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>44.21877224594726</v>
+        <v>34.21039601143217</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>12.64613769287738</v>
+        <v>18.25657600591554</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.3723816971104379</v>
+        <v>0.5235182400078677</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-1.376093206265457</v>
+        <v>-0.9161225546766618</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6655</v>
+        <v>6667</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>科定</t>
+          <t>信紘科</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>209.207742851952</v>
+        <v>210.7657977737905</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>118.5</v>
+        <v>257.5</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>49.49154175102331</v>
+        <v>44.21877224594726</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>7.156668259607301</v>
+        <v>12.64613769287738</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>2.20286052447702</v>
+        <v>0.3723816971104379</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.5787708837811114</v>
+        <v>-1.376093206265457</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6690</v>
+        <v>6655</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>安碁資訊</t>
+          <t>科定</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>203.7074948585973</v>
+        <v>209.207742851952</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>164</v>
+        <v>118.5</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,16 +6223,16 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>42.02058256651341</v>
+        <v>49.49154175102331</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>15.98714285281208</v>
+        <v>7.156668259607301</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.388873277849864</v>
+        <v>2.20286052447702</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.1960135610128901</v>
+        <v>0.5787708837811114</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6671</v>
+        <v>6690</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>三能-KY</t>
+          <t>安碁資訊</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>197.9365266232678</v>
+        <v>203.7074948585973</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>23.95</v>
+        <v>164</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,16 +6276,16 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>26.56520308604835</v>
+        <v>42.02058256651341</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>27.3177355463609</v>
+        <v>15.98714285281208</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>1.202865671940943</v>
+        <v>0.388873277849864</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.0552683644001045</v>
+        <v>-0.1960135610128901</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6715</v>
+        <v>6671</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>嘉基</t>
+          <t>三能-KY</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>194.3060506648899</v>
+        <v>197.9365266232678</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>411</v>
+        <v>23.95</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>46.46327996746811</v>
+        <v>26.56520308604835</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>14.90023299710576</v>
+        <v>27.3177355463609</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.80551933687569</v>
+        <v>1.202865671940943</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-8.870959085888012</v>
+        <v>0.0552683644001045</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6689</v>
+        <v>6715</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>伊雲谷</t>
+          <t>嘉基</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>188.7497681482161</v>
+        <v>194.3060506648899</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>63.2</v>
+        <v>411</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>41.8709490961181</v>
+        <v>46.46327996746811</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>15.80463341631883</v>
+        <v>14.90023299710576</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.2785968134938859</v>
+        <v>0.80551933687569</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.0715215503778678</v>
+        <v>-8.870959085888012</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6546</v>
+        <v>6689</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>正基</t>
+          <t>伊雲谷</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>185.6586573761158</v>
+        <v>188.7497681482161</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>64.2</v>
+        <v>63.2</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>36.49716696010616</v>
+        <v>41.8709490961181</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>17.05144356322627</v>
+        <v>15.80463341631883</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.2922161958339969</v>
+        <v>0.2785968134938859</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.593082558541727</v>
+        <v>0.0715215503778678</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6695</v>
+        <v>6546</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>芯鼎</t>
+          <t>正基</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>183.279232435053</v>
+        <v>185.6586573761158</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>56.3</v>
+        <v>64.2</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>49.93062921273379</v>
+        <v>36.49716696010616</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>16.66293454285049</v>
+        <v>17.05144356322627</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.6990974818544582</v>
+        <v>0.2922161958339969</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.6251969186733389</v>
+        <v>-0.593082558541727</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6763</v>
+        <v>6695</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>綠界科技</t>
+          <t>芯鼎</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>182.1786195236165</v>
+        <v>183.279232435053</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>43.4</v>
+        <v>56.3</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,16 +6541,16 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>36.04321721004237</v>
+        <v>49.93062921273379</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>18.96927453495573</v>
+        <v>16.66293454285049</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.3117525304616555</v>
+        <v>0.6990974818544582</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.4280653007389947</v>
+        <v>-0.6251969186733389</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6605</v>
+        <v>6763</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>帝寶</t>
+          <t>綠界科技</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>170.0415404476294</v>
+        <v>182.1786195236165</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>131</v>
+        <v>43.4</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,16 +6594,16 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>43.36504365513819</v>
+        <v>36.04321721004237</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>16.93848780614565</v>
+        <v>18.96927453495573</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>1.023378616534053</v>
+        <v>0.3117525304616555</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.954131633699155</v>
+        <v>-0.4280653007389947</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6552</v>
+        <v>6605</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>易華電</t>
+          <t>帝寶</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>166.2150451062504</v>
+        <v>170.0415404476294</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>27.4</v>
+        <v>131</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>39.09525624797468</v>
+        <v>43.36504365513819</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>13.31812990993144</v>
+        <v>16.93848780614565</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.5081692865779928</v>
+        <v>1.023378616534053</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.2941722273928475</v>
+        <v>-0.954131633699155</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6550</v>
+        <v>6552</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>北極星藥業-KY</t>
+          <t>易華電</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>147.5936988403236</v>
+        <v>166.2150451062504</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>12.8</v>
+        <v>27.4</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>42.54112745247213</v>
+        <v>39.09525624797468</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>20.29212535843526</v>
+        <v>13.31812990993144</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.4954937354678018</v>
+        <v>0.5081692865779928</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>0.0187186412840998</v>
+        <v>-0.2941722273928475</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6807</v>
+        <v>6550</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>峰源-KY</t>
+          <t>北極星藥業-KY</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>145.582233262222</v>
+        <v>147.5936988403236</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>33.45</v>
+        <v>12.8</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>48.10260701751763</v>
+        <v>42.54112745247213</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>11.08303326521074</v>
+        <v>20.29212535843526</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.5946296712571625</v>
+        <v>0.4954937354678018</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.06484597970777189</v>
+        <v>0.0187186412840998</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6558</v>
+        <v>6807</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>興能高</t>
+          <t>峰源-KY</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>140.9780244062702</v>
+        <v>145.582233262222</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>28.95</v>
+        <v>33.45</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>42.73870608386085</v>
+        <v>48.10260701751763</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.09145438424684</v>
+        <v>11.08303326521074</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.3796757668665679</v>
+        <v>0.5946296712571625</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.03640387357866</v>
+        <v>0.06484597970777189</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6720</v>
+        <v>6558</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>久昌</t>
+          <t>興能高</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>138.1183645580882</v>
+        <v>140.9780244062702</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>140</v>
+        <v>28.95</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>44.63680544953564</v>
+        <v>42.73870608386085</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>19.73982154257692</v>
+        <v>15.09145438424684</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.2664260971135668</v>
+        <v>0.3796757668665679</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.2595907218579674</v>
+        <v>-0.03640387357866</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6796</v>
+        <v>6720</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>晉弘</t>
+          <t>久昌</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>133.4008434170465</v>
+        <v>138.1183645580882</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>59</v>
+        <v>140</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,16 +6912,16 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>48.79160604687068</v>
+        <v>44.63680544953564</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>18.38738876697337</v>
+        <v>19.73982154257692</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.5596688037618257</v>
+        <v>0.2664260971135668</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L122" s="2" t="n">
         <v>0</v>
@@ -6930,31 +6930,31 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.3615804106386154</v>
+        <v>0.2595907218579674</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6614</v>
+        <v>6796</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>資拓宏宇</t>
+          <t>晉弘</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>105.1552084882685</v>
+        <v>133.4008434170465</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>39.05</v>
+        <v>59</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,13 +6965,13 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>39.88703534829151</v>
+        <v>48.79160604687068</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>19.0249712774154</v>
+        <v>18.38738876697337</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.3743461358409151</v>
+        <v>0.5596688037618257</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>0</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.0829676249250222</v>
+        <v>0.3615804106386154</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -6993,21 +6993,21 @@
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6838</v>
+        <v>6614</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>台新藥</t>
+          <t>資拓宏宇</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>97.7512658394015</v>
+        <v>105.1552084882685</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>24</v>
+        <v>39.05</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>43.97626731022017</v>
+        <v>39.88703534829151</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>10.79839316991049</v>
+        <v>19.0249712774154</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.3983339345955842</v>
+        <v>0.3743461358409151</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.0510026783589124</v>
+        <v>-0.0829676249250222</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7046,21 +7046,21 @@
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6771</v>
+        <v>6838</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>平和環保-創</t>
+          <t>台新藥</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>77.73646291062322</v>
+        <v>97.7512658394015</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>38.7</v>
+        <v>24</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>38.29743494748378</v>
+        <v>43.97626731022017</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>17.29262959025434</v>
+        <v>10.79839316991049</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.1230998787652709</v>
+        <v>0.3983339345955842</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.031143192891904</v>
+        <v>0.0510026783589124</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7099,21 +7099,21 @@
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>6597</v>
+        <v>6771</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>立誠</t>
+          <t>平和環保-創</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>62.13183839087929</v>
+        <v>77.73646291062322</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>66.7</v>
+        <v>38.7</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -7124,16 +7124,16 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>51.03943797591044</v>
+        <v>38.29743494748378</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>11.19706941299759</v>
+        <v>17.29262959025434</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>0.856814732783725</v>
+        <v>0.1230998787652709</v>
       </c>
       <c r="K126" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L126" s="2" t="n">
         <v>0</v>
@@ -7142,62 +7142,115 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>0.766709128704111</v>
+        <v>0.031143192891904</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
+        <v>6597</v>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>立誠</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>62.13183839087929</v>
+      </c>
+      <c r="E127" s="2" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
+        <v>51.03943797591044</v>
+      </c>
+      <c r="I127" s="2" t="n">
+        <v>11.19706941299759</v>
+      </c>
+      <c r="J127" s="2" t="n">
+        <v>0.856814732783725</v>
+      </c>
+      <c r="K127" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
+        <v>0.766709128704111</v>
+      </c>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>ema60_gt_ema120, market_above_ma60</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
         <v>6692</v>
       </c>
-      <c r="B127" s="2" t="inlineStr">
+      <c r="B128" s="2" t="inlineStr">
         <is>
           <t>進能服</t>
         </is>
       </c>
-      <c r="C127" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D127" s="2" t="n">
+      <c r="C128" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D128" s="2" t="n">
         <v>60.5795986414072</v>
       </c>
-      <c r="E127" s="2" t="n">
+      <c r="E128" s="2" t="n">
         <v>24.85</v>
       </c>
-      <c r="F127" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-16</t>
-        </is>
-      </c>
-      <c r="G127" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H127" s="2" t="n">
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H128" s="2" t="n">
         <v>42.57371745467325</v>
       </c>
-      <c r="I127" s="2" t="n">
+      <c r="I128" s="2" t="n">
         <v>11.92222093758873</v>
       </c>
-      <c r="J127" s="2" t="n">
+      <c r="J128" s="2" t="n">
         <v>0.260322792069474</v>
       </c>
-      <c r="K127" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L127" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M127" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N127" s="2" t="n">
+      <c r="K128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N128" s="2" t="n">
         <v>-0.0030650086963367</v>
       </c>
-      <c r="O127" s="2" t="inlineStr">
+      <c r="O128" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>